<commit_message>
Daily tables: add new hires of 19/10 and 20/10
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HsFNnGJRzg6EEfnut1VvMX
</commit_message>
<xml_diff>
--- a/loss-time/outputs/Nhap_lieu_05-10_den_20-10.xlsx
+++ b/loss-time/outputs/Nhap_lieu_05-10_den_20-10.xlsx
@@ -6057,7 +6057,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H39"/>
+  <dimension ref="A1:H41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -6815,12 +6815,12 @@
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>A2</t>
+          <t>P22</t>
         </is>
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>HC mới- 50% hiệu suất- 2 tuần-05/10</t>
+          <t>Đào tạo công nhân mới</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
@@ -6834,34 +6834,30 @@
         </is>
       </c>
       <c r="E22" s="5" t="n">
-        <v>0.3125</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="F22" s="5" t="n">
-        <v>0.5</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="G22" s="3" t="n">
-        <v>6</v>
-      </c>
-      <c r="H22" s="6" t="inlineStr">
-        <is>
-          <t>A2 ngày 12/12 - nhóm 05/10</t>
-        </is>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="H22" s="6" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>A2</t>
+          <t>P22</t>
         </is>
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>HC mới- 50% hiệu suất- 2 tuần-06/10</t>
+          <t>Đào tạo công nhân mới</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>Assembly</t>
+          <t>Machining</t>
         </is>
       </c>
       <c r="D23" s="3" t="inlineStr">
@@ -6870,19 +6866,15 @@
         </is>
       </c>
       <c r="E23" s="5" t="n">
-        <v>0.3125</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="F23" s="5" t="n">
-        <v>0.5</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="G23" s="3" t="n">
-        <v>7</v>
-      </c>
-      <c r="H23" s="6" t="inlineStr">
-        <is>
-          <t>A2 ngày 11/12 - nhóm 06/10</t>
-        </is>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="H23" s="6" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
@@ -6892,12 +6884,12 @@
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>HC mới- 50% hiệu suất- 2 tuần-06/10</t>
+          <t>HC mới- 50% hiệu suất- 2 tuần-05/10</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>Raw Cutting</t>
+          <t>Assembly</t>
         </is>
       </c>
       <c r="D24" s="3" t="inlineStr">
@@ -6912,11 +6904,11 @@
         <v>0.5</v>
       </c>
       <c r="G24" s="3" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H24" s="6" t="inlineStr">
         <is>
-          <t>A2 ngày 11/12 - nhóm 06/10</t>
+          <t>A2 ngày 12/12 - nhóm 05/10</t>
         </is>
       </c>
     </row>
@@ -6933,7 +6925,7 @@
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>Machining</t>
+          <t>Assembly</t>
         </is>
       </c>
       <c r="D25" s="3" t="inlineStr">
@@ -6948,7 +6940,7 @@
         <v>0.5</v>
       </c>
       <c r="G25" s="3" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="H25" s="6" t="inlineStr">
         <is>
@@ -6964,12 +6956,12 @@
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>HC mới- 50% hiệu suất- 2 tuần-07/10</t>
+          <t>HC mới- 50% hiệu suất- 2 tuần-06/10</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>Assembly</t>
+          <t>Raw Cutting</t>
         </is>
       </c>
       <c r="D26" s="3" t="inlineStr">
@@ -6984,11 +6976,11 @@
         <v>0.5</v>
       </c>
       <c r="G26" s="3" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H26" s="6" t="inlineStr">
         <is>
-          <t>A2 ngày 10/12 - nhóm 07/10</t>
+          <t>A2 ngày 11/12 - nhóm 06/10</t>
         </is>
       </c>
     </row>
@@ -7000,12 +6992,12 @@
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>HC mới- 50% hiệu suất- 2 tuần-07/10</t>
+          <t>HC mới- 50% hiệu suất- 2 tuần-06/10</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>Raw Cutting</t>
+          <t>Machining</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
@@ -7020,11 +7012,11 @@
         <v>0.5</v>
       </c>
       <c r="G27" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H27" s="6" t="inlineStr">
         <is>
-          <t>A2 ngày 10/12 - nhóm 07/10</t>
+          <t>A2 ngày 11/12 - nhóm 06/10</t>
         </is>
       </c>
     </row>
@@ -7036,12 +7028,12 @@
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>HC mới- 50% hiệu suất- 2 tuần-08/10</t>
+          <t>HC mới- 50% hiệu suất- 2 tuần-07/10</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>Raw Cutting</t>
+          <t>Assembly</t>
         </is>
       </c>
       <c r="D28" s="3" t="inlineStr">
@@ -7056,11 +7048,11 @@
         <v>0.5</v>
       </c>
       <c r="G28" s="3" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="H28" s="6" t="inlineStr">
         <is>
-          <t>A2 ngày 9/12 - nhóm 08/10</t>
+          <t>A2 ngày 10/12 - nhóm 07/10</t>
         </is>
       </c>
     </row>
@@ -7072,12 +7064,12 @@
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>HC mới- 50% hiệu suất- 2 tuần-08/10</t>
+          <t>HC mới- 50% hiệu suất- 2 tuần-07/10</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>Machining</t>
+          <t>Raw Cutting</t>
         </is>
       </c>
       <c r="D29" s="3" t="inlineStr">
@@ -7092,11 +7084,11 @@
         <v>0.5</v>
       </c>
       <c r="G29" s="3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H29" s="6" t="inlineStr">
         <is>
-          <t>A2 ngày 9/12 - nhóm 08/10</t>
+          <t>A2 ngày 10/12 - nhóm 07/10</t>
         </is>
       </c>
     </row>
@@ -7108,12 +7100,12 @@
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>HC mới- 50% hiệu suất- 2 tuần-09/10</t>
+          <t>HC mới- 50% hiệu suất- 2 tuần-08/10</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>Assembly</t>
+          <t>Raw Cutting</t>
         </is>
       </c>
       <c r="D30" s="3" t="inlineStr">
@@ -7128,11 +7120,11 @@
         <v>0.5</v>
       </c>
       <c r="G30" s="3" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="H30" s="6" t="inlineStr">
         <is>
-          <t>A2 ngày 8/12 - nhóm 09/10</t>
+          <t>A2 ngày 9/12 - nhóm 08/10</t>
         </is>
       </c>
     </row>
@@ -7144,12 +7136,12 @@
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>HC mới- 50% hiệu suất- 2 tuần-09/10</t>
+          <t>HC mới- 50% hiệu suất- 2 tuần-08/10</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>Raw Cutting</t>
+          <t>Machining</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
@@ -7164,11 +7156,11 @@
         <v>0.5</v>
       </c>
       <c r="G31" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H31" s="6" t="inlineStr">
         <is>
-          <t>A2 ngày 8/12 - nhóm 09/10</t>
+          <t>A2 ngày 9/12 - nhóm 08/10</t>
         </is>
       </c>
     </row>
@@ -7180,7 +7172,7 @@
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>HC mới- 50% hiệu suất- 2 tuần-12/10</t>
+          <t>HC mới- 50% hiệu suất- 2 tuần-09/10</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
@@ -7200,11 +7192,11 @@
         <v>0.5</v>
       </c>
       <c r="G32" s="3" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="H32" s="6" t="inlineStr">
         <is>
-          <t>A2 ngày 6/12 - nhóm 12/10</t>
+          <t>A2 ngày 8/12 - nhóm 09/10</t>
         </is>
       </c>
     </row>
@@ -7216,7 +7208,7 @@
       </c>
       <c r="B33" s="4" t="inlineStr">
         <is>
-          <t>HC mới- 50% hiệu suất- 2 tuần-12/10</t>
+          <t>HC mới- 50% hiệu suất- 2 tuần-09/10</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr">
@@ -7236,11 +7228,11 @@
         <v>0.5</v>
       </c>
       <c r="G33" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H33" s="6" t="inlineStr">
         <is>
-          <t>A2 ngày 6/12 - nhóm 12/10</t>
+          <t>A2 ngày 8/12 - nhóm 09/10</t>
         </is>
       </c>
     </row>
@@ -7252,7 +7244,7 @@
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t>HC mới- 50% hiệu suất- 2 tuần-13/10</t>
+          <t>HC mới- 50% hiệu suất- 2 tuần-12/10</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
@@ -7276,7 +7268,7 @@
       </c>
       <c r="H34" s="6" t="inlineStr">
         <is>
-          <t>A2 ngày 5/12 - nhóm 13/10</t>
+          <t>A2 ngày 6/12 - nhóm 12/10</t>
         </is>
       </c>
     </row>
@@ -7288,7 +7280,7 @@
       </c>
       <c r="B35" s="4" t="inlineStr">
         <is>
-          <t>HC mới- 50% hiệu suất- 2 tuần-13/10</t>
+          <t>HC mới- 50% hiệu suất- 2 tuần-12/10</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
@@ -7308,11 +7300,11 @@
         <v>0.5</v>
       </c>
       <c r="G35" s="3" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H35" s="6" t="inlineStr">
         <is>
-          <t>A2 ngày 5/12 - nhóm 13/10</t>
+          <t>A2 ngày 6/12 - nhóm 12/10</t>
         </is>
       </c>
     </row>
@@ -7329,7 +7321,7 @@
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>Machining</t>
+          <t>Assembly</t>
         </is>
       </c>
       <c r="D36" s="3" t="inlineStr">
@@ -7344,7 +7336,7 @@
         <v>0.5</v>
       </c>
       <c r="G36" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H36" s="6" t="inlineStr">
         <is>
@@ -7360,12 +7352,12 @@
       </c>
       <c r="B37" s="4" t="inlineStr">
         <is>
-          <t>HC mới- 50% hiệu suất- 2 tuần-14/10</t>
+          <t>HC mới- 50% hiệu suất- 2 tuần-13/10</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>Assembly</t>
+          <t>Raw Cutting</t>
         </is>
       </c>
       <c r="D37" s="3" t="inlineStr">
@@ -7380,11 +7372,11 @@
         <v>0.5</v>
       </c>
       <c r="G37" s="3" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H37" s="6" t="inlineStr">
         <is>
-          <t>A2 ngày 4/12 - nhóm 14/10</t>
+          <t>A2 ngày 5/12 - nhóm 13/10</t>
         </is>
       </c>
     </row>
@@ -7396,12 +7388,12 @@
       </c>
       <c r="B38" s="4" t="inlineStr">
         <is>
-          <t>HC mới- 50% hiệu suất- 2 tuần-15/10</t>
+          <t>HC mới- 50% hiệu suất- 2 tuần-13/10</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>Assembly</t>
+          <t>Machining</t>
         </is>
       </c>
       <c r="D38" s="3" t="inlineStr">
@@ -7416,11 +7408,11 @@
         <v>0.5</v>
       </c>
       <c r="G38" s="3" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H38" s="6" t="inlineStr">
         <is>
-          <t>A2 ngày 3/12 - nhóm 15/10</t>
+          <t>A2 ngày 5/12 - nhóm 13/10</t>
         </is>
       </c>
     </row>
@@ -7432,29 +7424,101 @@
       </c>
       <c r="B39" s="4" t="inlineStr">
         <is>
+          <t>HC mới- 50% hiệu suất- 2 tuần-14/10</t>
+        </is>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>Assembly</t>
+        </is>
+      </c>
+      <c r="D39" s="3" t="inlineStr">
+        <is>
+          <t>HR/ HSE</t>
+        </is>
+      </c>
+      <c r="E39" s="5" t="n">
+        <v>0.3125</v>
+      </c>
+      <c r="F39" s="5" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G39" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="H39" s="6" t="inlineStr">
+        <is>
+          <t>A2 ngày 4/12 - nhóm 14/10</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="3" t="inlineStr">
+        <is>
+          <t>A2</t>
+        </is>
+      </c>
+      <c r="B40" s="4" t="inlineStr">
+        <is>
+          <t>HC mới- 50% hiệu suất- 2 tuần-15/10</t>
+        </is>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>Assembly</t>
+        </is>
+      </c>
+      <c r="D40" s="3" t="inlineStr">
+        <is>
+          <t>HR/ HSE</t>
+        </is>
+      </c>
+      <c r="E40" s="5" t="n">
+        <v>0.3125</v>
+      </c>
+      <c r="F40" s="5" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G40" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="H40" s="6" t="inlineStr">
+        <is>
+          <t>A2 ngày 3/12 - nhóm 15/10</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="3" t="inlineStr">
+        <is>
+          <t>A2</t>
+        </is>
+      </c>
+      <c r="B41" s="4" t="inlineStr">
+        <is>
           <t>HC mới- 50% hiệu suất- 2 tuần-16/10</t>
         </is>
       </c>
-      <c r="C39" s="3" t="inlineStr">
+      <c r="C41" s="3" t="inlineStr">
         <is>
           <t>Assembly</t>
         </is>
       </c>
-      <c r="D39" s="3" t="inlineStr">
-        <is>
-          <t>HR/ HSE</t>
-        </is>
-      </c>
-      <c r="E39" s="5" t="n">
-        <v>0.3125</v>
-      </c>
-      <c r="F39" s="5" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="G39" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="H39" s="6" t="inlineStr">
+      <c r="D41" s="3" t="inlineStr">
+        <is>
+          <t>HR/ HSE</t>
+        </is>
+      </c>
+      <c r="E41" s="5" t="n">
+        <v>0.3125</v>
+      </c>
+      <c r="F41" s="5" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G41" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="H41" s="6" t="inlineStr">
         <is>
           <t>A2 ngày 2/12 - nhóm 16/10</t>
         </is>
@@ -7471,7 +7535,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H38"/>
+  <dimension ref="A1:H42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -8229,12 +8293,12 @@
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>A2</t>
+          <t>P22</t>
         </is>
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>HC mới- 50% hiệu suất- 2 tuần-06/10</t>
+          <t>Đào tạo công nhân mới</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
@@ -8248,34 +8312,30 @@
         </is>
       </c>
       <c r="E22" s="5" t="n">
-        <v>0.3125</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="F22" s="5" t="n">
-        <v>0.5</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="G22" s="3" t="n">
-        <v>7</v>
-      </c>
-      <c r="H22" s="6" t="inlineStr">
-        <is>
-          <t>A2 ngày 12/12 - nhóm 06/10</t>
-        </is>
-      </c>
+        <v>4</v>
+      </c>
+      <c r="H22" s="6" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>A2</t>
+          <t>P22</t>
         </is>
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>HC mới- 50% hiệu suất- 2 tuần-06/10</t>
+          <t>Đào tạo công nhân mới</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>Raw Cutting</t>
+          <t>Machining</t>
         </is>
       </c>
       <c r="D23" s="3" t="inlineStr">
@@ -8284,19 +8344,15 @@
         </is>
       </c>
       <c r="E23" s="5" t="n">
-        <v>0.3125</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="F23" s="5" t="n">
-        <v>0.5</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="G23" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="H23" s="6" t="inlineStr">
-        <is>
-          <t>A2 ngày 12/12 - nhóm 06/10</t>
-        </is>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="H23" s="6" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
@@ -8311,7 +8367,7 @@
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>Machining</t>
+          <t>Assembly</t>
         </is>
       </c>
       <c r="D24" s="3" t="inlineStr">
@@ -8326,7 +8382,7 @@
         <v>0.5</v>
       </c>
       <c r="G24" s="3" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="H24" s="6" t="inlineStr">
         <is>
@@ -8342,12 +8398,12 @@
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>HC mới- 50% hiệu suất- 2 tuần-07/10</t>
+          <t>HC mới- 50% hiệu suất- 2 tuần-06/10</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>Assembly</t>
+          <t>Raw Cutting</t>
         </is>
       </c>
       <c r="D25" s="3" t="inlineStr">
@@ -8362,11 +8418,11 @@
         <v>0.5</v>
       </c>
       <c r="G25" s="3" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H25" s="6" t="inlineStr">
         <is>
-          <t>A2 ngày 11/12 - nhóm 07/10</t>
+          <t>A2 ngày 12/12 - nhóm 06/10</t>
         </is>
       </c>
     </row>
@@ -8378,12 +8434,12 @@
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>HC mới- 50% hiệu suất- 2 tuần-07/10</t>
+          <t>HC mới- 50% hiệu suất- 2 tuần-06/10</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>Raw Cutting</t>
+          <t>Machining</t>
         </is>
       </c>
       <c r="D26" s="3" t="inlineStr">
@@ -8398,11 +8454,11 @@
         <v>0.5</v>
       </c>
       <c r="G26" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H26" s="6" t="inlineStr">
         <is>
-          <t>A2 ngày 11/12 - nhóm 07/10</t>
+          <t>A2 ngày 12/12 - nhóm 06/10</t>
         </is>
       </c>
     </row>
@@ -8414,12 +8470,12 @@
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>HC mới- 50% hiệu suất- 2 tuần-08/10</t>
+          <t>HC mới- 50% hiệu suất- 2 tuần-07/10</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>Raw Cutting</t>
+          <t>Assembly</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
@@ -8434,11 +8490,11 @@
         <v>0.5</v>
       </c>
       <c r="G27" s="3" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="H27" s="6" t="inlineStr">
         <is>
-          <t>A2 ngày 10/12 - nhóm 08/10</t>
+          <t>A2 ngày 11/12 - nhóm 07/10</t>
         </is>
       </c>
     </row>
@@ -8450,12 +8506,12 @@
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>HC mới- 50% hiệu suất- 2 tuần-08/10</t>
+          <t>HC mới- 50% hiệu suất- 2 tuần-07/10</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>Machining</t>
+          <t>Raw Cutting</t>
         </is>
       </c>
       <c r="D28" s="3" t="inlineStr">
@@ -8470,11 +8526,11 @@
         <v>0.5</v>
       </c>
       <c r="G28" s="3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H28" s="6" t="inlineStr">
         <is>
-          <t>A2 ngày 10/12 - nhóm 08/10</t>
+          <t>A2 ngày 11/12 - nhóm 07/10</t>
         </is>
       </c>
     </row>
@@ -8486,12 +8542,12 @@
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>HC mới- 50% hiệu suất- 2 tuần-09/10</t>
+          <t>HC mới- 50% hiệu suất- 2 tuần-08/10</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>Assembly</t>
+          <t>Raw Cutting</t>
         </is>
       </c>
       <c r="D29" s="3" t="inlineStr">
@@ -8506,11 +8562,11 @@
         <v>0.5</v>
       </c>
       <c r="G29" s="3" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="H29" s="6" t="inlineStr">
         <is>
-          <t>A2 ngày 9/12 - nhóm 09/10</t>
+          <t>A2 ngày 10/12 - nhóm 08/10</t>
         </is>
       </c>
     </row>
@@ -8522,12 +8578,12 @@
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>HC mới- 50% hiệu suất- 2 tuần-09/10</t>
+          <t>HC mới- 50% hiệu suất- 2 tuần-08/10</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>Raw Cutting</t>
+          <t>Machining</t>
         </is>
       </c>
       <c r="D30" s="3" t="inlineStr">
@@ -8542,11 +8598,11 @@
         <v>0.5</v>
       </c>
       <c r="G30" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H30" s="6" t="inlineStr">
         <is>
-          <t>A2 ngày 9/12 - nhóm 09/10</t>
+          <t>A2 ngày 10/12 - nhóm 08/10</t>
         </is>
       </c>
     </row>
@@ -8558,7 +8614,7 @@
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>HC mới- 50% hiệu suất- 2 tuần-12/10</t>
+          <t>HC mới- 50% hiệu suất- 2 tuần-09/10</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
@@ -8578,11 +8634,11 @@
         <v>0.5</v>
       </c>
       <c r="G31" s="3" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="H31" s="6" t="inlineStr">
         <is>
-          <t>A2 ngày 7/12 - nhóm 12/10</t>
+          <t>A2 ngày 9/12 - nhóm 09/10</t>
         </is>
       </c>
     </row>
@@ -8594,7 +8650,7 @@
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>HC mới- 50% hiệu suất- 2 tuần-12/10</t>
+          <t>HC mới- 50% hiệu suất- 2 tuần-09/10</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
@@ -8614,11 +8670,11 @@
         <v>0.5</v>
       </c>
       <c r="G32" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H32" s="6" t="inlineStr">
         <is>
-          <t>A2 ngày 7/12 - nhóm 12/10</t>
+          <t>A2 ngày 9/12 - nhóm 09/10</t>
         </is>
       </c>
     </row>
@@ -8630,7 +8686,7 @@
       </c>
       <c r="B33" s="4" t="inlineStr">
         <is>
-          <t>HC mới- 50% hiệu suất- 2 tuần-13/10</t>
+          <t>HC mới- 50% hiệu suất- 2 tuần-12/10</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr">
@@ -8654,7 +8710,7 @@
       </c>
       <c r="H33" s="6" t="inlineStr">
         <is>
-          <t>A2 ngày 6/12 - nhóm 13/10</t>
+          <t>A2 ngày 7/12 - nhóm 12/10</t>
         </is>
       </c>
     </row>
@@ -8666,7 +8722,7 @@
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t>HC mới- 50% hiệu suất- 2 tuần-13/10</t>
+          <t>HC mới- 50% hiệu suất- 2 tuần-12/10</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
@@ -8686,11 +8742,11 @@
         <v>0.5</v>
       </c>
       <c r="G34" s="3" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H34" s="6" t="inlineStr">
         <is>
-          <t>A2 ngày 6/12 - nhóm 13/10</t>
+          <t>A2 ngày 7/12 - nhóm 12/10</t>
         </is>
       </c>
     </row>
@@ -8707,7 +8763,7 @@
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>Machining</t>
+          <t>Assembly</t>
         </is>
       </c>
       <c r="D35" s="3" t="inlineStr">
@@ -8722,7 +8778,7 @@
         <v>0.5</v>
       </c>
       <c r="G35" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H35" s="6" t="inlineStr">
         <is>
@@ -8738,12 +8794,12 @@
       </c>
       <c r="B36" s="4" t="inlineStr">
         <is>
-          <t>HC mới- 50% hiệu suất- 2 tuần-14/10</t>
+          <t>HC mới- 50% hiệu suất- 2 tuần-13/10</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>Assembly</t>
+          <t>Raw Cutting</t>
         </is>
       </c>
       <c r="D36" s="3" t="inlineStr">
@@ -8758,11 +8814,11 @@
         <v>0.5</v>
       </c>
       <c r="G36" s="3" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H36" s="6" t="inlineStr">
         <is>
-          <t>A2 ngày 5/12 - nhóm 14/10</t>
+          <t>A2 ngày 6/12 - nhóm 13/10</t>
         </is>
       </c>
     </row>
@@ -8774,12 +8830,12 @@
       </c>
       <c r="B37" s="4" t="inlineStr">
         <is>
-          <t>HC mới- 50% hiệu suất- 2 tuần-15/10</t>
+          <t>HC mới- 50% hiệu suất- 2 tuần-13/10</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>Assembly</t>
+          <t>Machining</t>
         </is>
       </c>
       <c r="D37" s="3" t="inlineStr">
@@ -8794,11 +8850,11 @@
         <v>0.5</v>
       </c>
       <c r="G37" s="3" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H37" s="6" t="inlineStr">
         <is>
-          <t>A2 ngày 4/12 - nhóm 15/10</t>
+          <t>A2 ngày 6/12 - nhóm 13/10</t>
         </is>
       </c>
     </row>
@@ -8810,31 +8866,175 @@
       </c>
       <c r="B38" s="4" t="inlineStr">
         <is>
+          <t>HC mới- 50% hiệu suất- 2 tuần-14/10</t>
+        </is>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>Assembly</t>
+        </is>
+      </c>
+      <c r="D38" s="3" t="inlineStr">
+        <is>
+          <t>HR/ HSE</t>
+        </is>
+      </c>
+      <c r="E38" s="5" t="n">
+        <v>0.3125</v>
+      </c>
+      <c r="F38" s="5" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G38" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="H38" s="6" t="inlineStr">
+        <is>
+          <t>A2 ngày 5/12 - nhóm 14/10</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="3" t="inlineStr">
+        <is>
+          <t>A2</t>
+        </is>
+      </c>
+      <c r="B39" s="4" t="inlineStr">
+        <is>
+          <t>HC mới- 50% hiệu suất- 2 tuần-15/10</t>
+        </is>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>Assembly</t>
+        </is>
+      </c>
+      <c r="D39" s="3" t="inlineStr">
+        <is>
+          <t>HR/ HSE</t>
+        </is>
+      </c>
+      <c r="E39" s="5" t="n">
+        <v>0.3125</v>
+      </c>
+      <c r="F39" s="5" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G39" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="H39" s="6" t="inlineStr">
+        <is>
+          <t>A2 ngày 4/12 - nhóm 15/10</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="3" t="inlineStr">
+        <is>
+          <t>A2</t>
+        </is>
+      </c>
+      <c r="B40" s="4" t="inlineStr">
+        <is>
           <t>HC mới- 50% hiệu suất- 2 tuần-16/10</t>
         </is>
       </c>
-      <c r="C38" s="3" t="inlineStr">
+      <c r="C40" s="3" t="inlineStr">
         <is>
           <t>Assembly</t>
         </is>
       </c>
-      <c r="D38" s="3" t="inlineStr">
-        <is>
-          <t>HR/ HSE</t>
-        </is>
-      </c>
-      <c r="E38" s="5" t="n">
-        <v>0.3125</v>
-      </c>
-      <c r="F38" s="5" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="G38" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="H38" s="6" t="inlineStr">
+      <c r="D40" s="3" t="inlineStr">
+        <is>
+          <t>HR/ HSE</t>
+        </is>
+      </c>
+      <c r="E40" s="5" t="n">
+        <v>0.3125</v>
+      </c>
+      <c r="F40" s="5" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G40" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="H40" s="6" t="inlineStr">
         <is>
           <t>A2 ngày 3/12 - nhóm 16/10</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="3" t="inlineStr">
+        <is>
+          <t>A2</t>
+        </is>
+      </c>
+      <c r="B41" s="4" t="inlineStr">
+        <is>
+          <t>HC mới- 50% hiệu suất- 2 tuần-19/10</t>
+        </is>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>Assembly</t>
+        </is>
+      </c>
+      <c r="D41" s="3" t="inlineStr">
+        <is>
+          <t>HR/ HSE</t>
+        </is>
+      </c>
+      <c r="E41" s="5" t="n">
+        <v>0.3125</v>
+      </c>
+      <c r="F41" s="5" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G41" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="H41" s="6" t="inlineStr">
+        <is>
+          <t>A2 ngày 1/12 - nhóm 19/10</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="3" t="inlineStr">
+        <is>
+          <t>A2</t>
+        </is>
+      </c>
+      <c r="B42" s="4" t="inlineStr">
+        <is>
+          <t>HC mới- 50% hiệu suất- 2 tuần-19/10</t>
+        </is>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>Machining</t>
+        </is>
+      </c>
+      <c r="D42" s="3" t="inlineStr">
+        <is>
+          <t>HR/ HSE</t>
+        </is>
+      </c>
+      <c r="E42" s="5" t="n">
+        <v>0.3125</v>
+      </c>
+      <c r="F42" s="5" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G42" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="H42" s="6" t="inlineStr">
+        <is>
+          <t>A2 ngày 1/12 - nhóm 19/10</t>
         </is>
       </c>
     </row>

</xml_diff>